<commit_message>
actualizacion de modulo asistencia
</commit_message>
<xml_diff>
--- a/public/plantillas/reporte_confirmados.xlsx
+++ b/public/plantillas/reporte_confirmados.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\api_alcaldia_monteria\public\plantillas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\api_electoral\public\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7A596981-6BAE-4648-BF5D-A10D2AFCEF0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68BCA821-4ED5-4E94-ABC6-96D82D9F1A58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8EDF4DB8-0752-458A-8CE2-79743F0CC240}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t xml:space="preserve">PUESTO: </t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>OBSERVACION</t>
-  </si>
-  <si>
-    <t>COMANDO</t>
   </si>
   <si>
     <t>FECHA</t>
@@ -66,7 +63,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -80,6 +77,14 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -102,12 +107,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -126,9 +132,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -166,7 +172,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -272,7 +278,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -414,7 +420,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -422,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BC270BF-8467-483B-8DCE-8BC8EFCD7444}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.44140625" customWidth="1"/>
@@ -430,11 +436,10 @@
     <col min="3" max="3" width="40.109375" customWidth="1"/>
     <col min="4" max="4" width="6.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26.109375" customWidth="1"/>
-    <col min="6" max="6" width="23.5546875" customWidth="1"/>
-    <col min="7" max="7" width="20.88671875" customWidth="1"/>
+    <col min="6" max="6" width="20.88671875" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -442,7 +447,7 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -453,16 +458,13 @@
         <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>